<commit_message>
Gør udbytte-indtastning fleksibel: netto/brutto, manuel tabel og CSV
- Man kan nu angive ENTEN netto- eller bruttobeløb pr. udbyttelinje —
  det andet beregnes automatisk ud fra landets nettoprocent.
- Ny primær indgang: en redigerbar tabel (st.data_editor) hvor man
  indtaster direkte i UI'en, ingen fil nødvendig.
- Fil-upload er nu en genvej til at udfylde tabellen automatisk, og
  understøtter både Excel og CSV (med automatisk separator-detektion og
  dansk talformat som "18.823,41").
- Nyt eksempel: test_data/eksempel_udbytte.csv, samt opdateret .xlsx med
  en blanding af netto/brutto-rækker.
- Rettede en BOM-relateret kolonnegenkendelsesfejl i CSV-indlæsning.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199hXLLhFdNM4p9XUFugy97
</commit_message>
<xml_diff>
--- a/kursregulering/test_data/eksempel_udbytte.xlsx
+++ b/kursregulering/test_data/eksempel_udbytte.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,12 +429,17 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Beløb</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Dato</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Netto udbytte</t>
         </is>
       </c>
     </row>
@@ -451,12 +456,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2024-03-26</t>
+          <t>Netto</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>18823.41</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2024-03-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -471,11 +481,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Brutto</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>57823.2</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>2024-04-05</t>
         </is>
-      </c>
-      <c r="D3" t="n">
-        <v>49149.72</v>
       </c>
     </row>
     <row r="4">
@@ -491,12 +506,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2024-05-15</t>
+          <t>Netto</t>
         </is>
       </c>
       <c r="D4" t="n">
         <v>19489.99</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2024-05-15</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -509,6 +529,11 @@
           <t>DK</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Netto</t>
+        </is>
+      </c>
       <c r="D5" t="n">
         <v>6500</v>
       </c>
@@ -526,12 +551,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2024-06-01</t>
+          <t>Netto</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>2000</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2024-06-01</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -545,6 +575,11 @@
         </is>
       </c>
       <c r="C7" t="inlineStr">
+        <is>
+          <t>Netto</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>2024-07-01</t>
         </is>

</xml_diff>